<commit_message>
Sprint 5 Day 32: Added capital allocation reporting and validation
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M93"/>
+  <dimension ref="A1:V93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,51 @@
           <t>capex_lable</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern.1</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern.2</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern.3</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern.4</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern.5</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern.6</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern.7</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -529,6 +574,47 @@
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -568,6 +654,47 @@
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -615,6 +742,47 @@
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -662,6 +830,47 @@
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -709,6 +918,47 @@
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -756,6 +1006,47 @@
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -803,6 +1094,47 @@
       </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -850,6 +1182,47 @@
       </c>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -897,6 +1270,47 @@
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -928,6 +1342,31 @@
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -975,6 +1414,47 @@
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1022,6 +1502,43 @@
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1069,6 +1586,47 @@
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1116,6 +1674,47 @@
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1163,6 +1762,47 @@
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1210,6 +1850,47 @@
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1257,6 +1938,47 @@
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1304,6 +2026,47 @@
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1351,6 +2114,47 @@
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1398,6 +2202,47 @@
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1445,6 +2290,47 @@
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1492,6 +2378,47 @@
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1539,6 +2466,47 @@
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1586,6 +2554,47 @@
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1633,6 +2642,47 @@
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1680,6 +2730,47 @@
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1727,6 +2818,47 @@
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1774,6 +2906,47 @@
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1821,6 +2994,47 @@
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1868,6 +3082,47 @@
       </c>
       <c r="L31" t="inlineStr"/>
       <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1915,6 +3170,47 @@
       </c>
       <c r="L32" t="inlineStr"/>
       <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1962,6 +3258,47 @@
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2009,6 +3346,47 @@
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2056,6 +3434,47 @@
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2103,6 +3522,47 @@
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2150,6 +3610,47 @@
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2197,6 +3698,47 @@
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2244,6 +3786,47 @@
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2291,6 +3874,47 @@
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2334,6 +3958,47 @@
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2381,6 +4046,47 @@
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2428,6 +4134,47 @@
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2475,6 +4222,47 @@
       </c>
       <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2522,6 +4310,47 @@
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2569,6 +4398,47 @@
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2616,6 +4486,47 @@
       </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2663,6 +4574,47 @@
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2710,6 +4662,47 @@
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2757,6 +4750,47 @@
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2804,6 +4838,47 @@
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2851,6 +4926,47 @@
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2898,6 +5014,47 @@
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2945,6 +5102,47 @@
       </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2992,6 +5190,47 @@
       </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3037,6 +5276,47 @@
       </c>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3084,6 +5364,47 @@
       </c>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3131,6 +5452,47 @@
       </c>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3178,6 +5540,47 @@
       </c>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3225,6 +5628,47 @@
       </c>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3272,6 +5716,47 @@
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P61" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3319,6 +5804,47 @@
       </c>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3366,6 +5892,47 @@
       </c>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3413,6 +5980,47 @@
       </c>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3460,6 +6068,47 @@
       </c>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3507,6 +6156,47 @@
       </c>
       <c r="L66" t="inlineStr"/>
       <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3554,6 +6244,47 @@
       </c>
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3601,6 +6332,47 @@
       </c>
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3648,6 +6420,47 @@
       </c>
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3695,6 +6508,47 @@
       </c>
       <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3742,6 +6596,47 @@
       </c>
       <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3789,6 +6684,47 @@
       </c>
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3836,6 +6772,47 @@
       </c>
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3881,6 +6858,47 @@
       </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3928,6 +6946,47 @@
       </c>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3975,6 +7034,47 @@
       </c>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4022,6 +7122,47 @@
       </c>
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4069,6 +7210,47 @@
       </c>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4114,6 +7296,47 @@
       </c>
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4161,6 +7384,47 @@
       </c>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4208,6 +7472,47 @@
       </c>
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P81" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4255,6 +7560,31 @@
       </c>
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="O82" t="inlineStr"/>
+      <c r="P82" t="inlineStr"/>
+      <c r="Q82" t="inlineStr"/>
+      <c r="R82" t="inlineStr"/>
+      <c r="S82" t="inlineStr"/>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4302,6 +7632,47 @@
       </c>
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4349,6 +7720,47 @@
       </c>
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="P84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4396,6 +7808,47 @@
       </c>
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4443,6 +7896,47 @@
       </c>
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4490,6 +7984,47 @@
       </c>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4537,6 +8072,47 @@
       </c>
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="P88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4584,6 +8160,47 @@
       </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4631,6 +8248,47 @@
       </c>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4678,6 +8336,47 @@
       </c>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4725,6 +8424,47 @@
       </c>
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4772,6 +8512,47 @@
       </c>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>